<commit_message>
fix: explain missing basket indicators
</commit_message>
<xml_diff>
--- a/reports/investment_dashboard.xlsx
+++ b/reports/investment_dashboard.xlsx
@@ -12,9 +12,9 @@
     <sheet name="Reasons" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dashboard'!$A$3:$B$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dashboard'!$A$3:$B$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Key Indicators'!$A$1:$C$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Reasons'!$A$1:$B$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Reasons'!$A$1:$B$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -860,7 +860,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F13" s="2" t="n"/>
@@ -891,9 +891,7 @@
           <t>Risk Score</t>
         </is>
       </c>
-      <c r="B15" s="4" t="n">
-        <v>0</v>
-      </c>
+      <c r="B15" s="4" t="n"/>
       <c r="C15" s="2" t="n"/>
       <c r="D15" s="2" t="inlineStr">
         <is>
@@ -908,8 +906,16 @@
       <c r="F15" s="2" t="n"/>
     </row>
     <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="2" t="n"/>
-      <c r="B16" s="2" t="n"/>
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Missing Tickers</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>7747.HK, 000660.KS, 005930.KS, MU, MSFT, GOOGL, AMZN, META, AAPL, TSLA, QQQ, SOXX</t>
+        </is>
+      </c>
       <c r="C16" s="2" t="n"/>
       <c r="D16" s="2" t="inlineStr">
         <is>
@@ -960,9 +966,6 @@
           <t>Risk Score</t>
         </is>
       </c>
-      <c r="B19" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -993,7 +996,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:B15"/>
+  <autoFilter ref="A3:B16"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
@@ -1060,12 +1063,10 @@
           <t>Risk Score</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n">
-        <v>0</v>
-      </c>
+      <c r="B3" s="4" t="n"/>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -1190,7 +1191,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1249,8 +1250,56 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="4" t="n"/>
+      <c r="B6" s="8" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Data Quality Warnings</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Warning</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Fallback market data provider was used; review recommendation confidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Warning</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Missing market data for required tickers: 7747.HK, 000660.KS, 005930.KS, MU, MSFT, GOOGL, AMZN, META, AAPL, TSLA, QQQ, SOXX</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Warning</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Unavailable indicators due to insufficient source data: Relative Ratio, Risk Score, AI 5D Return, HBM 5D Return, D5, D20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B5"/>
+  <autoFilter ref="A1:B10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: show mobile proxy issue data in dashboard
</commit_message>
<xml_diff>
--- a/reports/investment_dashboard.xlsx
+++ b/reports/investment_dashboard.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dashboard'!$A$3:$B$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Key Indicators'!$A$1:$C$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Reasons'!$A$1:$B$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Reasons'!$A$1:$B$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Proxy Signal'!$A$1:$B$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -713,7 +713,7 @@
       <c r="C5" s="2" t="n"/>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Data quality is insufficient for a reliable basket decision.</t>
+          <t>Official equity data is incomplete.</t>
         </is>
       </c>
       <c r="E5" s="2" t="n"/>
@@ -727,13 +727,13 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>GitHub Issue</t>
+          <t>GitHub Issue Proxy</t>
         </is>
       </c>
       <c r="C6" s="2" t="n"/>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Missing required market data: 7747.HK, META, QQQ, SOXX</t>
+          <t>Tradable proxy data is used for intraday risk assessment only.</t>
         </is>
       </c>
       <c r="E6" s="2" t="n"/>
@@ -751,7 +751,11 @@
         </is>
       </c>
       <c r="C7" s="2" t="n"/>
-      <c r="D7" s="2" t="n"/>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Proxy data is not official equity market data.</t>
+        </is>
+      </c>
       <c r="E7" s="2" t="n"/>
       <c r="F7" s="2" t="n"/>
     </row>
@@ -767,7 +771,11 @@
         </is>
       </c>
       <c r="C8" s="2" t="n"/>
-      <c r="D8" s="2" t="n"/>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Proxy intraday risk level is Risk-On.</t>
+        </is>
+      </c>
       <c r="E8" s="2" t="n"/>
       <c r="F8" s="2" t="n"/>
     </row>
@@ -779,7 +787,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="C9" s="2" t="n"/>
@@ -810,7 +818,7 @@
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>64</v>
+        <v>12</v>
       </c>
       <c r="C11" s="2" t="n"/>
       <c r="D11" s="5" t="inlineStr">
@@ -828,7 +836,7 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>71.43000000000001</v>
+        <v>14.29</v>
       </c>
       <c r="C12" s="2" t="n"/>
       <c r="D12" s="2" t="inlineStr">
@@ -873,7 +881,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C14" s="2" t="n"/>
@@ -897,7 +905,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>binance+binance_proxy</t>
         </is>
       </c>
       <c r="C15" s="2" t="n"/>
@@ -921,7 +929,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Risk-On</t>
         </is>
       </c>
       <c r="C16" s="2" t="n"/>
@@ -945,7 +953,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="C17" s="2" t="n"/>
@@ -969,7 +977,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Uncertain</t>
+          <t>Cautious Hold</t>
         </is>
       </c>
       <c r="C18" s="2" t="n"/>
@@ -984,7 +992,7 @@
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>38</v>
+        <v>58</v>
       </c>
       <c r="C19" s="2" t="n"/>
       <c r="D19" s="2" t="n"/>
@@ -1097,7 +1105,7 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>7747.HK, META, QQQ, SOXX</t>
+          <t>7747.HK, 000660.KS, 005930.KS, MU, MSFT, GOOGL, AMZN, META, AAPL, TSLA, QQQ, SOXX</t>
         </is>
       </c>
       <c r="C27" s="2" t="n"/>
@@ -1371,7 +1379,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1406,7 +1414,7 @@
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>Data quality is insufficient for a reliable basket decision.</t>
+          <t>Official equity data is incomplete.</t>
         </is>
       </c>
     </row>
@@ -1416,45 +1424,41 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>Missing required market data: 7747.HK, META, QQQ, SOXX</t>
+          <t>Tradable proxy data is used for intraday risk assessment only.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="n"/>
-      <c r="B5" s="8" t="n"/>
+      <c r="A5" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Proxy data is not official equity market data.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Data Quality Warnings</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="inlineStr"/>
+      <c r="A6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Proxy intraday risk level is Risk-On.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Warning</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t>Fallback market data provider was used; review recommendation confidence.</t>
-        </is>
-      </c>
+      <c r="A7" s="4" t="n"/>
+      <c r="B7" s="8" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Warning</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>Missing market data for required tickers: 7747.HK, META, QQQ, SOXX</t>
-        </is>
-      </c>
+          <t>Data Quality Warnings</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -1464,7 +1468,7 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Recommendation is degraded because data quality is below the target.</t>
+          <t>Missing market data for required tickers: 7747.HK, 000660.KS, 005930.KS, MU, MSFT, GOOGL, AMZN, META, AAPL, TSLA, QQQ, SOXX</t>
         </is>
       </c>
     </row>
@@ -1476,7 +1480,7 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Manual mobile input was used from GitHub Issue on 2026-06-27.</t>
+          <t>Recommendation is degraded because data quality is below the target.</t>
         </is>
       </c>
     </row>
@@ -1488,12 +1492,36 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
+          <t>Manual mobile input was used from GitHub Issue Proxy on 2026-06-27.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Warning</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Tradable proxy price is not official equity market data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Warning</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
           <t>Unavailable indicators due to insufficient source data: Relative Ratio, Risk Score, AI 5D Return, HBM 5D Return, D5, D20</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B11"/>
+  <autoFilter ref="A1:B13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1531,7 +1559,7 @@
       </c>
       <c r="B2" s="8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1543,7 +1571,7 @@
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>binance+binance_proxy</t>
         </is>
       </c>
     </row>
@@ -1555,7 +1583,7 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>000660.KS, 005930.KS, AAPL, AMZN, GOOGL, META, MSFT, MU, NVDA, TSLA</t>
         </is>
       </c>
     </row>
@@ -1567,7 +1595,7 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>000660.KS: SKHYNIXUSDT, 005930.KS: SAMSUNGUSDT, AAPL: AAPLUSDT, AMZN: AMZNUSDT, GOOGL: GOOGLUSDT, META: METAUSDT, MSFT: MSFTUSDT, MU: MUUSDT, NVDA: NVDAUSDT, TSLA: TSLAUSDT</t>
         </is>
       </c>
     </row>
@@ -1577,7 +1605,9 @@
           <t>Proxy AI Change</t>
         </is>
       </c>
-      <c r="B6" s="8" t="n"/>
+      <c r="B6" s="8" t="n">
+        <v>2.146</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1585,7 +1615,9 @@
           <t>Proxy HBM Change</t>
         </is>
       </c>
-      <c r="B7" s="8" t="n"/>
+      <c r="B7" s="8" t="n">
+        <v>2.0802</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1595,7 +1627,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Risk-On</t>
         </is>
       </c>
     </row>
@@ -1607,7 +1639,7 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -1631,7 +1663,7 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor: switch AIOS to manual-only data mode
</commit_message>
<xml_diff>
--- a/reports/investment_dashboard.xlsx
+++ b/reports/investment_dashboard.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Key Indicators" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Reasons" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Proxy Signal" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="History Readiness" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dashboard'!$A$3:$B$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dashboard'!$A$3:$B$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Key Indicators'!$A$1:$C$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Reasons'!$A$1:$B$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Proxy Signal'!$A$1:$B$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Reasons'!$A$1:$B$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'History Readiness'!$A$1:$D$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -227,7 +227,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Dashboard'!B30</f>
+              <f>'Dashboard'!B26</f>
             </strRef>
           </tx>
           <spPr>
@@ -237,12 +237,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Dashboard'!$A$31:$A$36</f>
+              <f>'Dashboard'!$A$27:$A$32</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard'!$B$31:$B$36</f>
+              <f>'Dashboard'!$B$27:$B$32</f>
             </numRef>
           </val>
         </ser>
@@ -628,7 +628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -687,7 +687,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>csv</t>
+          <t>Manual Upload Only</t>
         </is>
       </c>
       <c r="C4" s="2" t="n"/>
@@ -702,7 +702,7 @@
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Manual Mobile Input Used</t>
+          <t>Manual Input Used</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -713,7 +713,7 @@
       <c r="C5" s="2" t="n"/>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Indicators do not align strongly enough for a directional mode.</t>
+          <t>Data quality is insufficient for a reliable basket decision.</t>
         </is>
       </c>
       <c r="E5" s="2" t="n"/>
@@ -727,13 +727,13 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>GitHub Issue</t>
+          <t>manual_upload</t>
         </is>
       </c>
       <c r="C6" s="2" t="n"/>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Conflicting signals favor watching instead of adjusting.</t>
+          <t>Insufficient manual history for 5D/Risk Score: 000660.KS, 005930.KS, AAPL, AMZN, GOOGL, META, MSFT, MU, TSLA. 5D requires at least 6 trading days.</t>
         </is>
       </c>
       <c r="E6" s="2" t="n"/>
@@ -751,11 +751,7 @@
         </is>
       </c>
       <c r="C7" s="2" t="n"/>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>Confidence is below the configured uncertainty threshold.</t>
-        </is>
-      </c>
+      <c r="D7" s="2" t="n"/>
       <c r="E7" s="2" t="n"/>
       <c r="F7" s="2" t="n"/>
     </row>
@@ -799,7 +795,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Fallback</t>
+          <t>Degraded</t>
         </is>
       </c>
       <c r="C10" s="2" t="n"/>
@@ -854,7 +850,7 @@
         </is>
       </c>
       <c r="B13" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C13" s="2" t="n"/>
       <c r="D13" s="2" t="inlineStr">
@@ -872,12 +868,12 @@
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Decision Influenced By Proxy</t>
+          <t>Today's Recommendation</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Uncertain</t>
         </is>
       </c>
       <c r="C14" s="2" t="n"/>
@@ -896,13 +892,11 @@
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Proxy Provider Used</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
+          <t>Confidence</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>38</v>
       </c>
       <c r="C15" s="2" t="n"/>
       <c r="D15" s="2" t="inlineStr">
@@ -920,12 +914,12 @@
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Proxy Risk Level</t>
+          <t>Risk Level</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="C16" s="2" t="n"/>
@@ -944,12 +938,12 @@
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Proxy Data Quality</t>
+          <t>Market Mode</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Mixed</t>
         </is>
       </c>
       <c r="C17" s="2" t="n"/>
@@ -968,13 +962,11 @@
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Today's Recommendation</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>Uncertain</t>
-        </is>
+          <t>Current Position</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>400</v>
       </c>
       <c r="C18" s="2" t="n"/>
       <c r="D18" s="2" t="n"/>
@@ -984,11 +976,11 @@
     <row r="19" ht="24" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Confidence</t>
+          <t>Suggested Position</t>
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>38</v>
+        <v>400</v>
       </c>
       <c r="C19" s="2" t="n"/>
       <c r="D19" s="2" t="n"/>
@@ -998,13 +990,11 @@
     <row r="20" ht="24" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Risk Level</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
+          <t>Position Delta</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="C20" s="2" t="n"/>
       <c r="D20" s="2" t="n"/>
@@ -1014,13 +1004,11 @@
     <row r="21" ht="24" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Market Mode</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>Mixed</t>
-        </is>
+          <t>Relative Ratio</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="n">
+        <v>0.4999343919862067</v>
       </c>
       <c r="C21" s="2" t="n"/>
       <c r="D21" s="2" t="n"/>
@@ -1030,12 +1018,10 @@
     <row r="22" ht="24" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Current Position</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="n">
-        <v>400</v>
-      </c>
+          <t>Risk Score</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="n"/>
       <c r="C22" s="2" t="n"/>
       <c r="D22" s="2" t="n"/>
       <c r="E22" s="2" t="n"/>
@@ -1044,11 +1030,13 @@
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Suggested Position</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="n">
-        <v>400</v>
+          <t>Missing Tickers</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
       </c>
       <c r="C23" s="2" t="n"/>
       <c r="D23" s="2" t="n"/>
@@ -1058,138 +1046,82 @@
     <row r="24" ht="24" customHeight="1">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Position Delta</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="n">
-        <v>0</v>
+          <t>Stale Tickers</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
       </c>
       <c r="C24" s="2" t="n"/>
       <c r="D24" s="2" t="n"/>
       <c r="E24" s="2" t="n"/>
       <c r="F24" s="2" t="n"/>
     </row>
-    <row r="25" ht="24" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Chart Metric</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
         <is>
           <t>Relative Ratio</t>
         </is>
       </c>
-      <c r="B25" s="4" t="n">
+      <c r="B27" t="n">
         <v>0.4999343919862067</v>
       </c>
-      <c r="C25" s="2" t="n"/>
-      <c r="D25" s="2" t="n"/>
-      <c r="E25" s="2" t="n"/>
-      <c r="F25" s="2" t="n"/>
-    </row>
-    <row r="26" ht="24" customHeight="1">
-      <c r="A26" s="3" t="inlineStr">
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
         <is>
           <t>Risk Score</t>
         </is>
       </c>
-      <c r="B26" s="4" t="n"/>
-      <c r="C26" s="2" t="n"/>
-      <c r="D26" s="2" t="n"/>
-      <c r="E26" s="2" t="n"/>
-      <c r="F26" s="2" t="n"/>
-    </row>
-    <row r="27" ht="24" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>Missing Tickers</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="n"/>
-      <c r="D27" s="2" t="n"/>
-      <c r="E27" s="2" t="n"/>
-      <c r="F27" s="2" t="n"/>
-    </row>
-    <row r="28" ht="24" customHeight="1">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>Stale Tickers</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="n"/>
-      <c r="D28" s="2" t="n"/>
-      <c r="E28" s="2" t="n"/>
-      <c r="F28" s="2" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>AI 5D Return</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Chart Metric</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Value</t>
+          <t>HBM 5D Return</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Relative Ratio</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>0.4999343919862067</v>
+          <t>D5</t>
+        </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Risk Score</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>AI 5D Return</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>HBM 5D Return</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>D5</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
           <t>D20</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:B28"/>
+  <autoFilter ref="A3:B24"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
-  <conditionalFormatting sqref="B5">
+  <conditionalFormatting sqref="B15">
     <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="0">
       <formula>70</formula>
     </cfRule>
@@ -1382,7 +1314,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1417,7 +1349,7 @@
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>Indicators do not align strongly enough for a directional mode.</t>
+          <t>Data quality is insufficient for a reliable basket decision.</t>
         </is>
       </c>
     </row>
@@ -1427,31 +1359,33 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>Conflicting signals favor watching instead of adjusting.</t>
+          <t>Insufficient manual history for 5D/Risk Score: 000660.KS, 005930.KS, AAPL, AMZN, GOOGL, META, MSFT, MU, TSLA. 5D requires at least 6 trading days.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="8" t="inlineStr">
-        <is>
-          <t>Confidence is below the configured uncertainty threshold.</t>
-        </is>
-      </c>
+      <c r="A5" s="4" t="n"/>
+      <c r="B5" s="8" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="n"/>
-      <c r="B6" s="8" t="n"/>
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Data Quality Warnings</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Data Quality Warnings</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="inlineStr"/>
+          <t>Warning</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Recommendation is degraded because data quality is below the target.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1461,7 +1395,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Fallback market data provider was used; review recommendation confidence.</t>
+          <t>Manual upload data was used from manual_upload on 2026-06-28.</t>
         </is>
       </c>
     </row>
@@ -1473,7 +1407,7 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Manual mobile input was used from GitHub Issue on 2026-06-28.</t>
+          <t>5D readiness is incomplete for 7747.HK, 000660.KS, 005930.KS, MU, MSFT, GOOGL, AMZN, META, AAPL, TSLA, QQQ, SOXX; at least 6 trading days are required.</t>
         </is>
       </c>
     </row>
@@ -1485,12 +1419,24 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
+          <t>20D readiness is incomplete for 7709.HK, 7747.HK, 000660.KS, 005930.KS, MU, NVDA, MSFT, GOOGL, AMZN, META, AAPL, TSLA, QQQ, SOXX; at least 21 trading days are required.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Warning</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
           <t>Unavailable indicators due to insufficient source data: Risk Score, AI 5D Return, HBM 5D Return, D5, D20</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B10"/>
+  <autoFilter ref="A1:B11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1501,32 +1447,52 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>Field</t>
+          <t>Ticker</t>
         </is>
       </c>
       <c r="B1" s="7" t="inlineStr">
         <is>
-          <t>Value</t>
+          <t>History Rows</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>5D Ready</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>20D Ready</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Available</t>
-        </is>
-      </c>
-      <c r="B2" s="8" t="inlineStr">
+          <t>000660.KS</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1535,86 +1501,158 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Provider Used</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>none</t>
+          <t>005930.KS</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Tickers Covered</t>
-        </is>
-      </c>
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>None</t>
+          <t>7709.HK</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Symbols Used</t>
-        </is>
-      </c>
-      <c r="B5" s="8" t="inlineStr">
-        <is>
-          <t>None</t>
+          <t>7747.HK</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Proxy AI Change</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="n"/>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Proxy HBM Change</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="n"/>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Proxy Risk Level</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>N/A</t>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Proxy Data Quality</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>Missing</t>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Official Conflict</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1623,10 +1661,18 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Decision Influenced</t>
-        </is>
-      </c>
-      <c r="B11" s="8" t="inlineStr">
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1635,17 +1681,85 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Warning</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>Tradable proxy price is not official equity market data.</t>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>SOXX</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B12"/>
+  <autoFilter ref="A1:D15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: show daily divergence and market cap ratio
</commit_message>
<xml_diff>
--- a/reports/investment_dashboard.xlsx
+++ b/reports/investment_dashboard.xlsx
@@ -13,9 +13,9 @@
     <sheet name="History Readiness" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dashboard'!$A$3:$B$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Key Indicators'!$A$1:$C$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Reasons'!$A$1:$B$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dashboard'!$A$3:$B$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Key Indicators'!$A$1:$C$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Reasons'!$A$1:$B$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'History Readiness'!$A$1:$D$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -227,7 +227,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Dashboard'!B26</f>
+              <f>'Dashboard'!B28</f>
             </strRef>
           </tx>
           <spPr>
@@ -237,12 +237,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Dashboard'!$A$27:$A$32</f>
+              <f>'Dashboard'!$A$29:$A$34</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard'!$B$27:$B$32</f>
+              <f>'Dashboard'!$B$29:$B$34</f>
             </numRef>
           </val>
         </ser>
@@ -628,7 +628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -855,7 +855,7 @@
       <c r="C13" s="2" t="n"/>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Risk Score</t>
+          <t>Samsung / SK Hynix Market Cap Ratio</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -879,7 +879,7 @@
       <c r="C14" s="2" t="n"/>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>AI 5D Return</t>
+          <t>Risk Score</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -901,12 +901,12 @@
       <c r="C15" s="2" t="n"/>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>HBM 5D Return</t>
+          <t>AI 1D Return</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0.1%</t>
         </is>
       </c>
       <c r="F15" s="2" t="n"/>
@@ -925,12 +925,12 @@
       <c r="C16" s="2" t="n"/>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>HBM 1D Return</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>-50.0%</t>
         </is>
       </c>
       <c r="F16" s="2" t="n"/>
@@ -949,12 +949,12 @@
       <c r="C17" s="2" t="n"/>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>D20</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>-50.1%</t>
         </is>
       </c>
       <c r="F17" s="2" t="n"/>
@@ -1059,65 +1059,102 @@
       <c r="E24" s="2" t="n"/>
       <c r="F24" s="2" t="n"/>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Chart Metric</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Relative Ratio</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>0.4999343919862067</v>
-      </c>
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Samsung / SK Hynix Market Cap Ratio</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="n"/>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="n"/>
+    </row>
+    <row r="26" ht="24" customHeight="1">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Market Cap Ratio Date</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="n"/>
+      <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="n"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Risk Score</t>
+          <t>Chart Metric</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Value</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>AI 5D Return</t>
-        </is>
+          <t>Relative Ratio</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>0.4999343919862067</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>HBM 5D Return</t>
+          <t>Samsung / SK Hynix Market Cap Ratio</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>Risk Score</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>D20</t>
-        </is>
+          <t>AI 1D Return</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>0.1025277360797494</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>HBM 1D Return</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>-49.95530365998058</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>-50.05783139606033</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:B24"/>
+  <autoFilter ref="A3:B26"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
@@ -1140,7 +1177,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1183,7 +1220,7 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Risk Score</t>
+          <t>Samsung / SK Hynix Market Cap Ratio</t>
         </is>
       </c>
       <c r="B3" s="4" t="n"/>
@@ -1196,7 +1233,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>AI 5D Return</t>
+          <t>Risk Score</t>
         </is>
       </c>
       <c r="B4" s="4" t="n"/>
@@ -1209,90 +1246,148 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>HBM 5D Return</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="n"/>
+          <t>AI 1D Return</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>0.1025277360797494</v>
+      </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0.1%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>D5</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="n"/>
+          <t>HBM 1D Return</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>-49.95530365998058</v>
+      </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>-50.0%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>D20</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="n"/>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>-50.05783139606033</v>
+      </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>-50.1%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>RSI14</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="n">
-        <v>100</v>
-      </c>
+          <t>AI 5D Return</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n"/>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>ADX14</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="n">
-        <v>100</v>
-      </c>
+          <t>HBM 5D Return</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n"/>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n"/>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>D20</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n"/>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>RSI14</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>ADX14</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
           <t>MACD</t>
         </is>
       </c>
-      <c r="B10" s="4" t="n">
+      <c r="B14" s="4" t="n">
         <v>12.09777575136146</v>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>12.10</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C10"/>
-  <conditionalFormatting sqref="B2:B10">
+  <autoFilter ref="A1:C14"/>
+  <conditionalFormatting sqref="B2:B14">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -1314,7 +1409,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1407,7 +1502,7 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>5D readiness is incomplete for 7747.HK, 000660.KS, 005930.KS, MU, MSFT, GOOGL, AMZN, META, AAPL, TSLA, QQQ, SOXX; at least 6 trading days are required.</t>
+          <t>Samsung / SK Hynix market cap ratio is unavailable; upload market_cap for both 005930.KS and 000660.KS in the same unit.</t>
         </is>
       </c>
     </row>
@@ -1419,7 +1514,7 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>20D readiness is incomplete for 7709.HK, 7747.HK, 000660.KS, 005930.KS, MU, NVDA, MSFT, GOOGL, AMZN, META, AAPL, TSLA, QQQ, SOXX; at least 21 trading days are required.</t>
+          <t>5D readiness is incomplete for 7747.HK, 000660.KS, 005930.KS, MU, MSFT, GOOGL, AMZN, META, AAPL, TSLA, QQQ, SOXX; at least 6 trading days are required.</t>
         </is>
       </c>
     </row>
@@ -1431,12 +1526,24 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Unavailable indicators due to insufficient source data: Risk Score, AI 5D Return, HBM 5D Return, D5, D20</t>
+          <t>20D readiness is incomplete for 7709.HK, 7747.HK, 000660.KS, 005930.KS, MU, NVDA, MSFT, GOOGL, AMZN, META, AAPL, TSLA, QQQ, SOXX; at least 21 trading days are required.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Warning</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Unavailable indicators due to insufficient source data: Samsung / SK Hynix Market Cap Ratio, Risk Score, AI 5D Return, HBM 5D Return, D5, D20</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B11"/>
+  <autoFilter ref="A1:B12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix: use manual daily changes for basket returns
</commit_message>
<xml_diff>
--- a/reports/investment_dashboard.xlsx
+++ b/reports/investment_dashboard.xlsx
@@ -838,7 +838,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>0.998</t>
         </is>
       </c>
       <c r="F12" s="2" t="n"/>
@@ -930,7 +930,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>-50.0%</t>
+          <t>-0.1%</t>
         </is>
       </c>
       <c r="F16" s="2" t="n"/>
@@ -954,7 +954,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>-50.1%</t>
+          <t>-0.2%</t>
         </is>
       </c>
       <c r="F17" s="2" t="n"/>
@@ -1008,7 +1008,7 @@
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>0.4999343919862067</v>
+        <v>0.9984765234765233</v>
       </c>
       <c r="C21" s="2" t="n"/>
       <c r="D21" s="2" t="n"/>
@@ -1108,7 +1108,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0.4999343919862067</v>
+        <v>0.9984765234765233</v>
       </c>
     </row>
     <row r="30">
@@ -1135,7 +1135,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>0.1025277360797494</v>
+        <v>0.1333333333333333</v>
       </c>
     </row>
     <row r="33">
@@ -1145,7 +1145,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>-49.95530365998058</v>
+        <v>-0.0525</v>
       </c>
     </row>
     <row r="34">
@@ -1155,7 +1155,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>-50.05783139606033</v>
+        <v>-0.1858333333333333</v>
       </c>
     </row>
   </sheetData>
@@ -1214,11 +1214,11 @@
         </is>
       </c>
       <c r="B2" s="4" t="n">
-        <v>0.4999343919862067</v>
+        <v>0.9984765234765233</v>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>0.998</t>
         </is>
       </c>
     </row>
@@ -1257,7 +1257,7 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>0.1025277360797494</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
@@ -1272,11 +1272,11 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>-49.95530365998058</v>
+        <v>-0.0525</v>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>-50.0%</t>
+          <t>-0.1%</t>
         </is>
       </c>
     </row>
@@ -1287,11 +1287,11 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>-50.05783139606033</v>
+        <v>-0.1858333333333333</v>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>-50.1%</t>
+          <t>-0.2%</t>
         </is>
       </c>
     </row>

</xml_diff>